<commit_message>
ETL V2 fix año
</commit_message>
<xml_diff>
--- a/reporte_Contactos.xlsx
+++ b/reporte_Contactos.xlsx
@@ -484,8 +484,8 @@
   <sheetFormatPr baseColWidth="8" defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="30" customWidth="1" style="5" min="1" max="1"/>
-    <col width="25" customWidth="1" style="5" min="2" max="2"/>
-    <col width="45" customWidth="1" style="5" min="3" max="3"/>
+    <col width="58.14" customWidth="1" style="5" min="2" max="2"/>
+    <col width="39.57" customWidth="1" style="5" min="3" max="3"/>
     <col width="53.29" customWidth="1" style="5" min="4" max="4"/>
     <col width="71.56999999999999" customWidth="1" style="5" min="5" max="5"/>
     <col width="41" customWidth="1" style="5" min="6" max="6"/>
@@ -507,7 +507,7 @@
         <is>
           <t>Empresa: BBVA
 Usuario: Uriel Meneses
-Fecha de descarga: 11-03-2026
+Fecha de descarga: 12-03-2026
 Descarga por Fecha de publicación del 2026-01-01 al 2026-01-31</t>
         </is>
       </c>

</xml_diff>